<commit_message>
menu perbaikan abensi dan pengajuan justifikasi
</commit_message>
<xml_diff>
--- a/public/assets/template_excel/template_unggah_absen_kehadiran_pegawai.xlsx
+++ b/public/assets/template_excel/template_unggah_absen_kehadiran_pegawai.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\neosimpeg\public\assets\template_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D8D59FB-C0F3-4DA7-A6BD-907F096D18B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912A0B20-C426-4EC3-9F24-BB8F7FEBB417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{91759EDF-54B6-43E9-84BB-C3F9C01EA305}"/>
   </bookViews>
@@ -41,15 +41,9 @@
     <t>nip</t>
   </si>
   <si>
-    <t>tgl mulai absen</t>
-  </si>
-  <si>
     <t>nama</t>
   </si>
   <si>
-    <t>tgl berakhir absen</t>
-  </si>
-  <si>
     <t>kode alasan absen</t>
   </si>
   <si>
@@ -57,6 +51,12 @@
   </si>
   <si>
     <t>tgl_sk</t>
+  </si>
+  <si>
+    <t>tgl mulai absen (d-m-Y)</t>
+  </si>
+  <si>
+    <t>tgl berakhir absen  (d-m-Y)</t>
   </si>
 </sst>
 </file>
@@ -414,8 +414,8 @@
   <cols>
     <col min="1" max="1" width="19.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.88671875" style="1"/>
     <col min="7" max="7" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
@@ -427,22 +427,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>